<commit_message>
Fix: Use valid UserRole enum and add missing username field to default user
</commit_message>
<xml_diff>
--- a/AirTrace_AI_Live_Data.xlsx
+++ b/AirTrace_AI_Live_Data.xlsx
@@ -176,25 +176,25 @@
     <t>Confidence Score</t>
   </si>
   <si>
-    <t>2026-07-20T16:13:28.224Z</t>
-  </si>
-  <si>
-    <t>90%</t>
-  </si>
-  <si>
-    <t>84%</t>
+    <t>2026-07-20T16:38:28.291Z</t>
+  </si>
+  <si>
+    <t>89%</t>
+  </si>
+  <si>
+    <t>91%</t>
+  </si>
+  <si>
+    <t>87%</t>
   </si>
   <si>
     <t>82%</t>
   </si>
   <si>
+    <t>86%</t>
+  </si>
+  <si>
     <t>83%</t>
-  </si>
-  <si>
-    <t>89%</t>
-  </si>
-  <si>
-    <t>86%</t>
   </si>
   <si>
     <t>Traffic Contribution (%)</t>
@@ -815,7 +815,7 @@
         <v>19</v>
       </c>
       <c r="N2" s="2">
-        <v>427</v>
+        <v>396</v>
       </c>
       <c r="O2" s="2">
         <v>85</v>
@@ -862,7 +862,7 @@
         <v>22</v>
       </c>
       <c r="N3" s="2">
-        <v>327</v>
+        <v>309</v>
       </c>
       <c r="O3" s="2">
         <v>87</v>
@@ -909,7 +909,7 @@
         <v>25</v>
       </c>
       <c r="N4" s="2">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="O4" s="2">
         <v>73</v>
@@ -956,7 +956,7 @@
         <v>28</v>
       </c>
       <c r="N5" s="2">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="O5" s="2">
         <v>48</v>
@@ -1003,7 +1003,7 @@
         <v>31</v>
       </c>
       <c r="N6" s="2">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="O6" s="2">
         <v>61</v>
@@ -1050,7 +1050,7 @@
         <v>25</v>
       </c>
       <c r="N7" s="2">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="O7" s="2">
         <v>67</v>
@@ -1097,7 +1097,7 @@
         <v>36</v>
       </c>
       <c r="N8" s="2">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="O8" s="2">
         <v>54</v>
@@ -1144,7 +1144,7 @@
         <v>31</v>
       </c>
       <c r="N9" s="2">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="O9" s="2">
         <v>52</v>
@@ -1191,7 +1191,7 @@
         <v>19</v>
       </c>
       <c r="N10" s="2">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="O10" s="2">
         <v>45</v>
@@ -1238,7 +1238,7 @@
         <v>43</v>
       </c>
       <c r="N11" s="2">
-        <v>230</v>
+        <v>262</v>
       </c>
       <c r="O11" s="2">
         <v>49</v>
@@ -1285,7 +1285,7 @@
         <v>46</v>
       </c>
       <c r="N12" s="2">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="O12" s="2">
         <v>75</v>
@@ -1332,7 +1332,7 @@
         <v>49</v>
       </c>
       <c r="N13" s="2">
-        <v>298</v>
+        <v>322</v>
       </c>
       <c r="O13" s="2">
         <v>71</v>
@@ -1383,7 +1383,7 @@
         <v>412</v>
       </c>
       <c r="D2" s="2">
-        <v>427</v>
+        <v>396</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>54</v>
@@ -1400,7 +1400,7 @@
         <v>319</v>
       </c>
       <c r="D3" s="2">
-        <v>327</v>
+        <v>309</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>55</v>
@@ -1417,10 +1417,10 @@
         <v>288</v>
       </c>
       <c r="D4" s="2">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1434,10 +1434,10 @@
         <v>185</v>
       </c>
       <c r="D5" s="2">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1451,10 +1451,10 @@
         <v>205</v>
       </c>
       <c r="D6" s="2">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1468,10 +1468,10 @@
         <v>178</v>
       </c>
       <c r="D7" s="2">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1485,10 +1485,10 @@
         <v>144</v>
       </c>
       <c r="D8" s="2">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1502,10 +1502,10 @@
         <v>237</v>
       </c>
       <c r="D9" s="2">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1519,10 +1519,10 @@
         <v>246</v>
       </c>
       <c r="D10" s="2">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1536,10 +1536,10 @@
         <v>240</v>
       </c>
       <c r="D11" s="2">
-        <v>230</v>
+        <v>262</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1553,7 +1553,7 @@
         <v>191</v>
       </c>
       <c r="D12" s="2">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>59</v>
@@ -1570,10 +1570,10 @@
         <v>307</v>
       </c>
       <c r="D13" s="2">
-        <v>298</v>
+        <v>322</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1727,7 +1727,7 @@
         <v>26</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1750,7 +1750,7 @@
         <v>26</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1773,7 +1773,7 @@
         <v>40</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1796,7 +1796,7 @@
         <v>19</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1842,7 +1842,7 @@
         <v>22</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>